<commit_message>
Add 6 edge-case rows to the test data; fix two bugs they exposed
- Workbook: WEB-014 (web quote form, feet, CFA), EML-022 (numbers in
  words), EML-023 (color tie during an open quote), EML-024 (no
  quantity), EML-025 (discontinued), EML-026 (pending trade review);
  marked in a Notes column and the Read Me tab; original kept in
  case-study-prompt/
- Fix: an ambiguous line no longer supersedes an open quote
- Fix: a pending trade review isn't bypassed, and AI-vs-rules
  disagreement on an unknown sender goes to review
- Tests for every added row (36 total); docs note the data decision

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/perennials_sample_data.xlsx
+++ b/data/perennials_sample_data.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18000" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fabric Catalog" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing Rules" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Existing CRM Records" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inbound Requests" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fabric Catalog" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Pricing Rules" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Existing CRM Records" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Inbound Requests" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fabric Catalog'!$A$1:$H$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pricing Rules'!$A$1:$C$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Existing CRM Records'!$A$1:$G$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Inbound Requests'!$A$1:$H$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Inbound Requests'!$A$1:$I$28</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -463,7 +463,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -478,7 +477,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -514,11 +512,17 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
           <t>Available yards = Yards On Hand − Yards Reserved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Added for testing: rows WEB-014 and EML-022 to EML-026 are not in the original case-study data. They cover edge cases the original rows don't (see the Notes column). The original file is in case-study-prompt/.</t>
         </is>
       </c>
     </row>
@@ -1915,7 +1919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1926,6 +1930,7 @@
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
     <col width="70" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1969,6 +1974,11 @@
           <t>Message</t>
         </is>
       </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -2820,8 +2830,286 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>WEB-014</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Quote request</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Website form</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-21 09:15</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Mara Lowe</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Mara Lowe Design</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>mara@maralowedesign.example</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Sidemark: LOWE / Malibu living room.</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Added for testing (not in the original case-study data): the site's Request A Quote form: 90 feet, Date Needed, CFA requested (lines in web_cart_submissions.json).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>EML-022</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Quote request</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-21 11:40</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Tom Becker</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Brightwater Yacht Interiors</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>tbecker@brightwateryi.example</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Following up on the swatches for the yacht: the grey mesh is perfect. We'll need sixty yards of it, and the same of the white canvas.</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>Added for testing (not in the original case-study data): quantities written as words. Rules can't read them (draft a question); Claude can (they disagree, so review).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>EML-023</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Quote request</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-21 14:05</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Mara Lowe</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Mara Lowe Design</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>mara@maralowedesign.example</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Can I also get 10 yds of the linen for the window seat?</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Added for testing (not in the original case-study data): real color tie (she sampled Sand and Charcoal) while a linen quote is open; must ask, not revise the open quote.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>EML-024</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Quote request</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:50</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Sam Hollis</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Hollis &amp; Park Architects</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>shollis@hollispark.example</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>Could you price the plaid for the booths too?</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>Added for testing (not in the original case-study data): no quantity: draft one question instead of guessing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>EML-025</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Quote request</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-22 13:30</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Kevin Ortiz</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Ortiz Upholstery Co.</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>kevin@ortizupholstery.example</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>My customer is set on the Sunset Ikat for the dining chairs after all. Can you quote 30 yds and hold it?</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Added for testing (not in the original case-study data): discontinued fabric: quote only the 22 yd that remain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>EML-026</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Quote request</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-23 10:10</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Hannah Kim</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr"/>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>hannahkim.home@gmail.example</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>Hi again! While you look at my samples, could you price 20 yds of the garnet velvet?</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>Added for testing (not in the original case-study data): quote from a sender whose trade status isn't verified yet (WEB-012 still in review).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H22"/>
+  <autoFilter ref="A1:I28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>